<commit_message>
Save CF's dxfs to the styles part
The test file file for MaintainConditionalFormattingOrder is updated
with a new styles part and few other changes. No semantic change.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Other/StyleReferenceFiles/ConditionalFormattingOrder/ConditionalFormattingOrder.xlsx
+++ b/ClosedXML.Tests/Resource/Other/StyleReferenceFiles/ConditionalFormattingOrder/ConditionalFormattingOrder.xlsx
@@ -20,99 +20,93 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="0" uniqueCount="0"/>
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac x16r2">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="0" formatCode=""/>
-  </x:numFmts>
-  <x:fonts count="3" x14ac:knownFonts="1">
-    <x:font>
-      <x:sz val="11"/>
-      <x:color theme="1"/>
-      <x:name val="等线"/>
-      <x:family val="2"/>
-      <x:scheme val="minor"/>
-    </x:font>
-    <x:font>
-      <x:sz val="9"/>
-      <x:name val="等线"/>
-      <x:family val="3"/>
-      <x:charset val="134"/>
-      <x:scheme val="minor"/>
-    </x:font>
-    <x:font>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="2">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-  </x:fills>
-  <x:borders count="1">
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-      <x:diagonal/>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </x:cellStyleXfs>
-  <x:cellXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="常规" xfId="0" builtinId="0"/>
-  </x:cellStyles>
-  <x:dxfs count="3">
-    <x:dxf>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:fgColor auto="1"/>
-          <x:bgColor theme="9"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:fgColor auto="1"/>
-          <x:bgColor rgb="FFFFFF00"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:fgColor auto="1"/>
-          <x:bgColor rgb="FFFF0000"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-  </x:dxfs>
-  <x:tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <x:extLst>
-    <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="5">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </x:ext>
-    <x:ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
       <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </x:ext>
-  </x:extLst>
-</x:styleSheet>
+    </ext>
+  </extLst>
+</styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -392,13 +386,13 @@
   </x:sheetData>
   <x:phoneticPr fontId="1" type="noConversion"/>
   <x:conditionalFormatting sqref="A1:A1">
-    <x:cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="greaterThan">
+    <x:cfRule type="cellIs" dxfId="2" priority="1" stopIfTrue="1" operator="greaterThan">
       <x:formula>5</x:formula>
     </x:cfRule>
-    <x:cfRule type="cellIs" dxfId="1" priority="2" stopIfTrue="1" operator="greaterThan">
+    <x:cfRule type="cellIs" dxfId="0" priority="2" stopIfTrue="1" operator="greaterThan">
       <x:formula>2</x:formula>
     </x:cfRule>
-    <x:cfRule type="cellIs" dxfId="2" priority="3" stopIfTrue="1" operator="greaterThan">
+    <x:cfRule type="cellIs" dxfId="1" priority="3" stopIfTrue="1" operator="greaterThan">
       <x:formula>0</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>

</xml_diff>